<commit_message>
fix: update literature review fields
</commit_message>
<xml_diff>
--- a/literature_review_results/v6_annotator1_opencoding.xlsx
+++ b/literature_review_results/v6_annotator1_opencoding.xlsx
@@ -8,19 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mjavadmt\Desktop\EnergySmell\LiteratureReviewResults\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4998FB-B629-4528-8C39-544043BB81E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594F1CF3-F6DE-47C1-8EEF-CA73C790C13C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="taxonomy" sheetId="3" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">taxonomy!$A$1:$F$77</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1291" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1735" uniqueCount="873">
   <si>
     <t>Pattern</t>
   </si>
@@ -2022,12 +2026,690 @@
   <si>
     <t>Unpredictable branches</t>
   </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Parent_ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>Work is executed that does not contribute to the required observable output or is executed more often than needed or only adds to the computation time. This category covers wasted CPU time from statements, calls, and setup that can be removed or deferred without changing required behavior. Also, unoptimized path which delays reaching to output and forces unnecessary wrok with extra copmutation overhead. Also, sometimes declaring or copying which adds unnecessary computation and can be optimized, can be considered here. Use this category when the main issue is that the work should not have been done at all (or at that frequency), not that it was done with the wrong data structure or algorithm.</t>
+  </si>
+  <si>
+    <t>C1.S1</t>
+  </si>
+  <si>
+    <t>Subcategory</t>
+  </si>
+  <si>
+    <t>Computes values or performs calls whose results are never used on any required execution path. This includes calculations stored to variables that are never read, or helper calls whose return values are ignored. Do not use this label when the work is required for side effects such as necessary I/O, required logging, or synchronization.</t>
+  </si>
+  <si>
+    <t>Example: Building a list of transformed items and then never returning or consuming it; calling a heavy function and storing it in a variable but never using that variable.</t>
+  </si>
+  <si>
+    <t>C1.S2</t>
+  </si>
+  <si>
+    <t>Executes statements that leave program state unchanged or repeat an idempotent action without need. Typical signals include assignments like x = x, repeated casts that do not change the value, or repeated resets to the same value. Applying a function to a variable when the transformation does not meaningfully change the outcome for the intended task can be redundant. Avoid using this label when repetition is required for correctness due to external state changes.</t>
+  </si>
+  <si>
+    <t>Example: Repeatedly converting an integer to int() inside a loop when it is already an int; performing x = x in a hot path, or for example, if your goal is to find the maximum element of a list, applying a softmax to the list first is unnecessary, since softmax preserves the ordering of elements, the index of the maximum value remains the same.</t>
+  </si>
+  <si>
+    <t>C1.S3</t>
+  </si>
+  <si>
+    <t>Performs setup, initialization, or calculations on execution paths where the result is not required (e.g., before an early return) or is immediately overwritten or can be done more efficiently later.</t>
+  </si>
+  <si>
+    <t>Example: Creating an empty list at the top of a function on every call even when most calls return early before using it.</t>
+  </si>
+  <si>
+    <t>C1.S4</t>
+  </si>
+  <si>
+    <t>Invokes expensive runtime/housekeeping operations more often than needed, such as forcing garbage collection, flushing buffers, or manual compaction. These calls can dominate CPU time and disrupt normal runtime optimizations. Use this label when the call frequency itself is the waste (even if the call has side effects).</t>
+  </si>
+  <si>
+    <t>Example: Calling GC.collect() (or an equivalent) repeatedly inside a loop; forcing disk flush after every small write without a correctness requirement.</t>
+  </si>
+  <si>
+    <t>C1.S5</t>
+  </si>
+  <si>
+    <t>Unnecessarily copying some object into another object, which the new copied object is used in the rest of the execution path, however, the object is not changing or the change to the object does not matter. In this case, copying only added extra overhead</t>
+  </si>
+  <si>
+    <t>Example: Copying an entire list before read-only iteration when the original list is not mutated by the loop.</t>
+  </si>
+  <si>
+    <t>C1.S6</t>
+  </si>
+  <si>
+    <t>By simplifying the input before applying a heavy operation, we can reduce redundant computation and reach the result faster and more efficiently.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example: doing (x * 0) + (y * 1) instead of simplyfying it first. </t>
+  </si>
+  <si>
+    <t>C1.S7</t>
+  </si>
+  <si>
+    <t>When two functions A and B can be applied in any order and produce the same final result (i.e., A(B(x))=B(A(x))), the order of execution can still significantly impact performance. Choosing the less efficient order may increase total computation time by performing unnecessary work or processing more data than needed. In some cases, this is equivalent to taking a longer path to reach the same output.</t>
+  </si>
+  <si>
+    <t>Example: doing sorting and then taking the numbers less than 100 , instead of getting numbers less than 100 first and then sorting.</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>Extra layers of calls, wrappers, delegation, or dispatch add overhead without providing required modularity or behavior. This category is about CPU cost from call/return, stack frames, binding/dispatch, and wrapper logic. Use it when the same work could be performed directly with equivalent semantics and safety.</t>
+  </si>
+  <si>
+    <t>C2.S1</t>
+  </si>
+  <si>
+    <t>Delegates a simple operation to another method purely for abstraction in a hot path, adding call/return overhead without functional benefit. Signals include many small one-line methods that immediately forward to another method. It can also be calling internal accesor like getters/setters or wrapper access internally when direct field access would be equivalent and safe. This adds call overhead and sometimes repeated validation work. Do not label as a smell when the boundary is required for API stability, testing seams, or real polymorphic behavior.</t>
+  </si>
+  <si>
+    <t>Example: A hot function calls helperA(), which only calls helperB() and returns its result, with no validation or alternate behavior.</t>
+  </si>
+  <si>
+    <t>C2.S2</t>
+  </si>
+  <si>
+    <t>Uses instance methods or dynamic dispatch when the operation does not depend on instance state or subtype behavior. This forces extra binding/dispatch and may require loading object context unnecessarily. This is distinct from method delegation: here the issue is dispatch/binding cost, not an extra wrapper layer. Do not use when the behavior truly varies by subtype or needs instance state.</t>
+  </si>
+  <si>
+    <t>Example: Defining a helper as an instance method even though it never references self/this, causing per-call binding overhead.</t>
+  </si>
+  <si>
+    <t>C2.S3</t>
+  </si>
+  <si>
+    <t>Splits a performance-critical flow into too many tiny layers (methods, wrappers, indirections) that each add overhead, even if each layer does 'something'. The hallmark is high call depth and frequent small transitions in tight loops or frequently executed paths. This differs from unnecessary method delegation because each layer may perform small logic; the issue is the cumulative structural overhead. Do not label when the decomposition is required for correctness, security boundaries, or genuinely reusable interfaces.</t>
+  </si>
+  <si>
+    <t>Example: A tight loop that calls several thin wrappers (validate→normalize→convert→dispatch) per element, where these could be fused without changing required behavior.</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>Iteration performs more per-iteration work than necessary or uses an avoidably costly traversal form. This category covers inefficiencies amplified by unfiltered bulk iteration, missed early exits, loop-invariant work kept inside loops, and avoidable nested loops. Use this label when the primary driver is how work is repeated across iterations, not a wrong overall algorithm or wrong data structure.</t>
+  </si>
+  <si>
+    <t>C3.S1</t>
+  </si>
+  <si>
+    <t>Processes all items even though only a subset, window, or top-k is needed for the required output. The distinguishing feature is that the loop's domain is larger than required, not that the body is expensive. Do not use when a full pass is required (e.g., global aggregation, full validation).</t>
+  </si>
+  <si>
+    <t>Example: When only first 10 items of list is required to be mapped to 2 * x, however you iterate over all items, even though you only update the first 10.</t>
+  </si>
+  <si>
+    <t>C3.S2</t>
+  </si>
+  <si>
+    <t>Continues iterating after the required result has already been determined. Signals include searches that find the answer but keep scanning, or loops that could short-circuit but do not. Do not use when the loop must continue for required side effects (e.g., writing every element).</t>
+  </si>
+  <si>
+    <t>Example: After finding a target item in a list, the loop continues processing remaining items even though only the first match is required.</t>
+  </si>
+  <si>
+    <t>C3.S3</t>
+  </si>
+  <si>
+    <t>Recomputes values inside the loop that are constant across iterations (length checks, repeated lookups, repeated conversions, repeated function results). The key is that the recomputed value would be identical if computed once before the loop or cached.</t>
+  </si>
+  <si>
+    <t>Example: Calling len(list) or list.size() in the loop condition each iteration; repeatedly compiling the same regex inside the loop body.</t>
+  </si>
+  <si>
+    <t>C3.S4</t>
+  </si>
+  <si>
+    <t>Uses an iteration form with avoidable overhead, such as manual indexing when direct iteration is available and equivalent. This can introduce extra bounds checks, repeated indexing operations, or more complex control flow. This differs from loop-invariant recomputation: the overhead comes from the traversal mechanism itself. Do not use when indexing is required (needs index values, parallel arrays).</t>
+  </si>
+  <si>
+    <t>Example: Iterating over a list with `for i in range(len(a))` and repeatedly indexing `a[i]` when `for x in a` is sufficient.</t>
+  </si>
+  <si>
+    <t>C3.S5</t>
+  </si>
+  <si>
+    <t>Uses nested loops where an equivalent approach reduces complexity (e.g., quadratic to linear/log-linear) or avoids redundant pair checks. The primary signal is avoidable O(N^2) or worse behavior caused by looping structure. Or for example, we can decrease from n^2 to n(n+1)/2. Do not use when the problem is inherently quadratic and inputs are provably tiny.</t>
+  </si>
+  <si>
+    <t>Example: checking if two numbers summation would be equal to a target number. We can inefficiently do n^2 if we process earlier item from our index. Because the earlier item and current index has been checked before in the previous loop. So we should do it in triangular upper matrix search rather than full matrix search.</t>
+  </si>
+  <si>
+    <t>C3.S6</t>
+  </si>
+  <si>
+    <t>Creates expensive objects or performs heavy initialization inside a loop when it could be hoisted, reused, or bulk-initialized. This includes defining functions inside loops, allocating large buffers repeatedly, or constructing helper structures each iteration.</t>
+  </si>
+  <si>
+    <t>Example: Initializing a new large list/array inside every iteration; defining a helper function inside a loop body instead of once outside.</t>
+  </si>
+  <si>
+    <t>C3.S7</t>
+  </si>
+  <si>
+    <t>Modifies the same sequence being iterated (inserts/removes/reorders), which can trigger repeated shifting, reindexing, or skipped elements. This often causes hidden quadratic behavior and can also introduce subtle correctness bugs. Do not use when the language/structure guarantees safe in-place iteration without extra work and it is measured to be negligible.</t>
+  </si>
+  <si>
+    <t>Example: Removing items from a Python list while looping over it, causing elements to shift and the loop to do extra work or skip items.</t>
+  </si>
+  <si>
+    <t>C3.S8</t>
+  </si>
+  <si>
+    <t>Loop unrolling is a code optimization technique that duplicates the body of a loop multiple times to reduce the overhead of branch instructions and counter increments. By decreasing these control statements, it creates longer sequences of "straight-line" code that allow the CPU to process instructions more efficiently.</t>
+  </si>
+  <si>
+    <t>Example: Standard Loop: A loop that performs one addition, then checks if it should stop, repeating this cycle 100 times.
+Unrolled Loop: A loop that performs four additions in a row before checking if it should stop, repeating this cycle only 25 times to reach the same total.</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>Branching performs extra checks or uses an evaluation structure that increases expected runtime cost. This category includes poor short-circuit ordering, redundant or constant conditions, deep nesting that prevents early returns, and expensive control-flow mechanisms like exceptions. Use it when the inefficiency is driven by how decisions are evaluated, not by data structures or loops.</t>
+  </si>
+  <si>
+    <t>C4.S1</t>
+  </si>
+  <si>
+    <t>Orders AND/OR conditions so expensive checks run more often than necessary. For AND chains, cheap/likely-false checks should typically come first; for OR chains, cheap/likely-true checks should come first. Do not reorder when it changes semantics due to side effects or exceptions.</t>
+  </si>
+  <si>
+    <t>Example: `if expensive_check(x) and x is not None:` instead of checking `x is not None` first.</t>
+  </si>
+  <si>
+    <t>C4.S2</t>
+  </si>
+  <si>
+    <t>Evaluates conditions that are always true/false in the relevant context, or repeats a check already implied by earlier logic. The defining feature is that the extra check cannot change the control outcome. Here the redundancy is logical, not structural. Do not use when conditions are controlled by required configuration flags and the overhead is not on the hot path.</t>
+  </si>
+  <si>
+    <t>Example: Checking `x != None` twice in the same branch path; testing a flag that is always true in the deployed configuration. Or for example when you know some number is always greater than zero, but you again check that if number is greater than zero (calling abs(x) on it).</t>
+  </si>
+  <si>
+    <t>C4.S3</t>
+  </si>
+  <si>
+    <t>Uses multiple independent `if` statements when branches are mutually exclusive, causing extra evaluations. The key signal is that at most one branch can execute, but the code tests multiple conditions anyway. This differs from deep nesting: the issue is repeated checks, not readability structure. Do not use when multiple branches may legitimately execute.</t>
+  </si>
+  <si>
+    <t>Example: Three separate `if` blocks checking ranges of the same value, where an `if/elif/else` chain would stop after the first match.</t>
+  </si>
+  <si>
+    <t>C4.S4</t>
+  </si>
+  <si>
+    <t>Uses nested conditionals that prevent early returns and cause repeated checks or unnecessary execution of inner blocks. A guard clause can often return early to skip the rest of the logic. Do not use when nesting is necessary and does not add repeated evaluation or extra work.</t>
+  </si>
+  <si>
+    <t>Example: Multiple nested `if` blocks that only gate access to a final simple operation, instead of returning early when a precondition fails.</t>
+  </si>
+  <si>
+    <t>C4.S5</t>
+  </si>
+  <si>
+    <t>Uses higher-cost precision, reflection, or runtime type introspection when a cheaper equivalent meets requirements. The hallmark is that the decision could be made with simpler types or polymorphism without changing correctness. Do not use when precision/type checking is required by the spec or safety constraints.</t>
+  </si>
+  <si>
+    <t>Example: Using reflection/isinstance checks inside a tight loop instead of relying on a common interface; using high-precision float comparisons when integer/boolean checks suffice.</t>
+  </si>
+  <si>
+    <t>C4.S6</t>
+  </si>
+  <si>
+    <t>Uses exceptions (try/except) as the normal way to select between expected outcomes. Raising and handling exceptions typically allocates exception objects and unwinds stack frames, which is far more expensive than simple conditional checks. Do not use when exceptions represent truly exceptional/error conditions and occur rarely.</t>
+  </si>
+  <si>
+    <t>Example: Attempting a dictionary lookup and catching KeyError on the common path instead of checking membership when misses are frequent.</t>
+  </si>
+  <si>
+    <t>C4.S7</t>
+  </si>
+  <si>
+    <t>Fails to check trivial or common edge cases that would allow skipping heavy computation. The defining feature is that a small, cheap pre-check at the top would bypass an expensive path for many inputs. Do not use when the edge case is extremely rare or the guard check would itself be expensive.</t>
+  </si>
+  <si>
+    <t>Example: Not checking for empty or single-element input before running a full sort or complex processing pipeline that is unnecessary for those cases.</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Energy waste caused by choosing or introducing data structures or representations that increase compute or memory pressure for the required operations. This includes wrong container choice, missing helper structures, unnecessary intermediate structures, and overly heavy representations for simple values. Use this category when the main issue is the *shape* or *type* of data used for the task.</t>
+  </si>
+  <si>
+    <t>C5.S1</t>
+  </si>
+  <si>
+    <t>Uses a structure with worse asymptotic or constant-factor behavior for the required operations when constraints do not demand it. The key signal is a mismatch between operation needs (membership, random access, ordering) and the chosen structure. Do not use when ordering/stability/memory constraints legitimately justify the choice.</t>
+  </si>
+  <si>
+    <t>Example: Using a list for frequent membership tests when a set would give O(1) lookups and ordering is not required Or Using a standard list to manage a queue where elements are frequently removed from the front, forcing the CPU to shift every remaining item in memory for each operation</t>
+  </si>
+  <si>
+    <t>C5.S2</t>
+  </si>
+  <si>
+    <t>Fails to introduce an auxiliary structure that would reduce repeated cost, such as an index map, set for membership, or precomputed lookup. Use this label when building the helper once enables faster repeated operations over a dataset. Do not use when the helper construction cost exceeds the benefit (very small N or single use).</t>
+  </si>
+  <si>
+    <t>Example: Repeatedly scanning a list to find matching IDs instead of building a dict/map from ID to object once. Or Repeatedly scanning a 10,000-character string to count the occurrences of each letter, resulting in millions of redundant comparisons. By introducing an intermediate "frequency map" (dictionary) to store counts in a single pass, the total work is reduced to a linear $O(n)$ operation.</t>
+  </si>
+  <si>
+    <t>C5.S3</t>
+  </si>
+  <si>
+    <t>Introduces an intermediate structure or converts between representations without necessity. The defining feature is that the data could remain in its original form for the required operations, or the transformation could be done once and reused. The extra container or conversion exists only for convenience or coding style, but adds avoidable compute or memory overhead. Creating intermediate containers that are not required (e.g., materializing a list only to iterate once).
+Repeated or avoidable format conversions (e.g., string ↔ object, JSON ↔ dict, tensor ↔ list) when the data could stay in one representation.</t>
+  </si>
+  <si>
+    <t>Example: Converting a generator to a list only to iterate once, when direct iteration over the generator is sufficient.</t>
+  </si>
+  <si>
+    <t>C5.S4</t>
+  </si>
+  <si>
+    <t>Chooses a heavier type/representation than required for the value’s constraints, increasing memory and compute cost. This includes using boxed/wrapper primitives instead of primitives, or using large/complex types for small fixed-size values. The issue is the chosen type/representation, not allocating too much capacity. Do not use when the heavier representation is required by interfaces, interoperability, or correctness guarantees.</t>
+  </si>
+  <si>
+    <t>Example: Storing a single-character value as a full string object where a character/byte type is available and sufficient, or using float when value is always int.</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>Patterns that allocate, copy, retain, or leak memory beyond what is required, increasing GC pressure and energy cost. This category focuses on memory churn and retention. Use it when the primary issue is that too much data is created or kept alive, not merely accessed inefficiently. If the memory pressure comes from an external resource not released, this category includes that as resource leakage.</t>
+  </si>
+  <si>
+    <t>C6.S1</t>
+  </si>
+  <si>
+    <t>Copies large objects/arrays when a reference, view, slice, or in-place update is sufficient. The key signal is duplicated memory with identical content created solely to proceed with computation. Do not use when defensive copies are required for correctness or immutability guarantees.</t>
+  </si>
+  <si>
+    <t>C6.S2</t>
+  </si>
+  <si>
+    <t>Unnecessary data materialization is when you create and store intermediate data (like lists or tables) even though you don’t need to keep it.
+It wastes memory and computation when the data could be processed directly or lazily instead.</t>
+  </si>
+  <si>
+    <t>Example: Reading a whole file into memory with read() when line-by-line streaming processing is sufficient. For example:
+numbers = [1, 2, 3, 4, 5]
+squared = [x*x for x in numbers]   # creates a full new list in memory
+total = sum(squared)</t>
+  </si>
+  <si>
+    <t>C6.S3</t>
+  </si>
+  <si>
+    <t>Keeps whole structures when smaller or compressed or optimized representations would suffice for downstream operations. The signal is that large objects stay alive long after only small parts are needed. Do not use when later operations truly need the full object frequently.</t>
+  </si>
+  <si>
+    <t>Example: Storing entire substrings or full objects when storing indices/IDs and fetching on demand would meet requirements.</t>
+  </si>
+  <si>
+    <t>C6.S4</t>
+  </si>
+  <si>
+    <t>Allocates larger buffers/containers than needed for typical inputs, increasing memory footprint and cache/GC pressure. The hallmark is consistently low utilization of allocated capacity. Do not use when extra capacity is deliberately used to reduce reallocations in a proven hotspot.</t>
+  </si>
+  <si>
+    <t>Example: Allocating a very large fixed-size buffer for small strings or small messages, leading to wasted memory.</t>
+  </si>
+  <si>
+    <t>C6.S5</t>
+  </si>
+  <si>
+    <t>Fails to release external resources promptly (files, sockets, DB connections), causing memory and resource bloat over time. This can also keep associated buffers and internal runtime objects alive, increasing energy use. Use this label when proper closing/disposal would prevent ongoing retention.</t>
+  </si>
+  <si>
+    <t>Example: Opening database connections in a loop without closing them; leaving file handles open across many requests.</t>
+  </si>
+  <si>
+    <t>C6.S6</t>
+  </si>
+  <si>
+    <t>Uses a mutable object (e.g., list/dict) as a default parameter value so it is allocated once and then shared across calls. This can unintentionally retain data, grow over time, and create surprising cross-call coupling that increases memory and processing cost. Do not use when the pattern is intentionally used as a measured, correctly managed cache and is documented.</t>
+  </si>
+  <si>
+    <t>Example: `def f(x, acc=[]): acc.append(x); return acc` causing the same list to grow across calls and consume more memory.</t>
+  </si>
+  <si>
+    <t>C6.S7</t>
+  </si>
+  <si>
+    <t>Declaring a variable that occupies significant space in the memory that can be removed as it has no effect on the execution path. It can also reflect cases where the variable is used in the execution pathes, but its usage is unnecessary and can be replaced with direct values.</t>
+  </si>
+  <si>
+    <t>Example: defining a new variable every time after each computation where you do not need the intermediate results and occupies space; or, defining var x which is not used in the execution path at all and takes space.</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>Energy waste from choosing a strategy or algorithm that explores more of the problem than needed. This category is about fundamental complexity (Big-O) or systematic extra work across the problem space. Use it when fixing local code patterns (loops/conditions) is not enough because the overall approach is inefficient.</t>
+  </si>
+  <si>
+    <t>C7.S1</t>
+  </si>
+  <si>
+    <t>Uses an algorithm with known worse complexity or higher constant factors for the same required result when a better alternative exists. The key signal is that a different standard approach would reduce runtime across typical input sizes. Do not use when inputs are guaranteed tiny and the overhead of a 'better' algorithm dominates.</t>
+  </si>
+  <si>
+    <t>Example: Using a naive sorting approach in a hot path when a library sort or a linear-time selection algorithm would meet requirements.</t>
+  </si>
+  <si>
+    <t>C7.S2</t>
+  </si>
+  <si>
+    <t>Explores a large space of possibilities exhaustively without applying constraints or pruning early. The hallmark is exponential or very large search work that grows quickly with input size. Do not use when completeness requires brute force and the search space is provably small.</t>
+  </si>
+  <si>
+    <t>Example: Trying every possible combination of parameters even though simple bounds checks could discard most candidates early.</t>
+  </si>
+  <si>
+    <t>C7.S3</t>
+  </si>
+  <si>
+    <t>Computes results for parts of the problem that do not affect the final output. The key signal is that a cheaper, more direct computation exists that avoids full processing. Do not use when the 'extra' results are required for later features or correctness.</t>
+  </si>
+  <si>
+    <t>Example: Sorting an entire list to find the maximum element, when a single linear scan would produce the same required output.</t>
+  </si>
+  <si>
+    <t>C7.S4</t>
+  </si>
+  <si>
+    <t>Re-solves overlapping subproblems as part of the overall strategy, common in naive recursion or repeated searches. The hallmark is repeated evaluation of the same logical subcases across the computation.</t>
+  </si>
+  <si>
+    <t>Example: A recursive function recomputes the same intermediate results for many branches instead of storing them once.</t>
+  </si>
+  <si>
+    <t>C7.S5</t>
+  </si>
+  <si>
+    <t>Uses recursion where an iterative solution is straightforward, adding repeated function-call overhead and risking stack overflow. The energy cost comes from deep call stacks and repeated prologue/epilogue work.</t>
+  </si>
+  <si>
+    <t>Example: Computing a simple cumulative sum via recursion over a list instead of a single iterative loop.</t>
+  </si>
+  <si>
+    <t>C7.S6</t>
+  </si>
+  <si>
+    <t>Explores subproblems in an order that delays pruning or delays finding an early solution, increasing expected work. The defining feature is that reordering decisions (while preserving correctness) would reduce explored states on average. Do not use when ordering cannot be changed safely due to correctness constraints.</t>
+  </si>
+  <si>
+    <t>Example: In constraint search, expanding the least-constrained variable first, causing far more backtracking than choosing the most-constrained variable early.</t>
+  </si>
+  <si>
+    <t>C8</t>
+  </si>
+  <si>
+    <t>Energy waste from failing to reuse results of expensive computations or lookups. This includes memoization of deterministic functions, reuse of derived/prepared artifacts, and local caching of repeated accesses in hot code. Use it when the same value is computed or retrieved multiple times and could be stored and reused without changing required semantics.</t>
+  </si>
+  <si>
+    <t>C8.S1</t>
+  </si>
+  <si>
+    <t>Recomputes deterministic expensive function results for identical inputs instead of caching and reusing them. The hallmark is repeated calls with the same arguments producing the same output. Do not use when inputs rarely repeat or caching would violate memory constraints.</t>
+  </si>
+  <si>
+    <t>Example: Recomputing an expensive parse/analysis function for the same string key many times across a request, instead of caching the result.</t>
+  </si>
+  <si>
+    <t>C8.S2</t>
+  </si>
+  <si>
+    <t>Recreates expensive derived artifacts (parsed forms, compiled patterns, prepared queries, initialized models) instead of reusing them. The key signal is that the derived object could be built once and used many times with the same semantics. Do not use when the derived artifact depends on frequently changing configuration or inputs.</t>
+  </si>
+  <si>
+    <t>Example: Compiling the same regular expression on every call rather than compiling once and reusing it.</t>
+  </si>
+  <si>
+    <t>C8.S3</t>
+  </si>
+  <si>
+    <t>Repeatedly performs chained property/attribute/member access in hot code instead of caching intermediate references locally. The key feature is repeated dereferencing of the same chain where intermediate objects do not change. Do not use when intermediate objects legitimately change each iteration.</t>
+  </si>
+  <si>
+    <t>Example: Inside a loop, repeatedly reading `obj.a.b.c.d` when `tmp = obj.a.b.c` can be cached once and `tmp.d` reused.</t>
+  </si>
+  <si>
+    <t>C8.S4</t>
+  </si>
+  <si>
+    <t>Repeatedly retrieving the same static or slowly changing data from an external source (DB, File, API) instead of buffering it locally.</t>
+  </si>
+  <si>
+    <t>Example: while you have loaded the file into current variable, you still load the file again.</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>Inefficiencies in transferring, retrieving, or persisting data between the application and external systems (disk, network, database, APIs). These costs are often dominated by latency, serialization, and round-trip overhead, so reducing call count and transferred bytes is critical. Use this category when the primary cost is crossing system boundaries or traversing layered data sources.</t>
+  </si>
+  <si>
+    <t>C9.S1</t>
+  </si>
+  <si>
+    <t>Performs many small I/O operations instead of batching into fewer larger operations. Typical signals include line-by-line writes with flushes, per-item network calls, or N+1 database query patterns. Do not use when the protocol truly requires per-item round trips (rare) and cannot be redesigned.</t>
+  </si>
+  <si>
+    <t>Example: Issuing one database query per row in a loop instead of fetching rows in a single batched query.</t>
+  </si>
+  <si>
+    <t>C9.S2</t>
+  </si>
+  <si>
+    <t>Fetches or sends more data than is actually consumed by the logic, increasing bandwidth, parsing, and memory cost. Signals include SELECT * when only a few columns are needed, reading full files when only headers are used, or sending full objects instead of IDs/ranges. Do not use when partial transfer/compression is unavailable or would increase CPU cost more than it saves.</t>
+  </si>
+  <si>
+    <t>Example: Downloading full records including large blobs when only a small identifier and timestamp are needed.</t>
+  </si>
+  <si>
+    <t>C9.S3</t>
+  </si>
+  <si>
+    <t>Requires multiple dependent retrieval steps to find the needed data (fetch A to locate B to locate C), with substantial processing at each hop. This pattern often appears in layered database access or object graphs with repeated lookups. Refactoring typically provides direct access paths, denormalization, or caching of the final mapping.</t>
+  </si>
+  <si>
+    <t>Example: Querying one table to get IDs, then querying another table for each ID, then querying a third table for each of those results.</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>Energy waste from not using available optimized language features, standard libraries, or bulk/vectorized primitives. This category applies when equivalent semantics can be achieved with a more efficient built-in or library routine (often implemented in lower-level code). Also, if someone uses unnecessary built-in functions which could be solved easily without that this case can be applied.</t>
+  </si>
+  <si>
+    <t>C10.S1</t>
+  </si>
+  <si>
+    <t>Manually implements functionality that is provided by a highly optimized built-in or standard library function. The hallmark is custom loops or manual logic that replicates common operations like sorting, searching, counting, or aggregation. Do not use when custom behavior is required and built-ins cannot express the needed semantics.</t>
+  </si>
+  <si>
+    <t>Example: Writing a manual min/max scan with extra overhead where a built-in `min()`/`max()` (or language equivalent) is available and sufficient.</t>
+  </si>
+  <si>
+    <t>C10.S2</t>
+  </si>
+  <si>
+    <t>Chooses a built-in/library tool that is semantically equivalent but more expensive than a simpler alternative. The key signal is unnecessary features or generality that you do not use (extra parsing, extra allocations, heavier data types). Do not use when the extra features are truly required by the task.</t>
+  </si>
+  <si>
+    <t>Using re.match('^prefix', s) (Regular Expressions) to check if dynamic string s starts with a literal value, instead of using the lighter s.startswith('prefix')</t>
+  </si>
+  <si>
+    <t>C10.S3</t>
+  </si>
+  <si>
+    <t>Uses per-element operations where a bulk/batched/vectorized primitive exists with equivalent results. The hallmark is repeated API calls inside loops that could be replaced by one bulk call that reduces overhead and improves locality. This differs from fragmented I/O (Category 9): here the calls are in-process APIs (or batchable library operations), not necessarily external round trips. Do not use when bulk APIs change ordering, atomicity, or semantics you rely on.</t>
+  </si>
+  <si>
+    <t>Example: Appending one element at a time with costly conversions when a bulk `extend`, `join`, or vectorized library call can process the whole collection.</t>
+  </si>
+  <si>
+    <t>C10.S4</t>
+  </si>
+  <si>
+    <t>Builds strings via repeated concatenation, especially in loops, causing repeated allocations and copying as strings are immutable in many languages. The key signal is O(N^2)-like behavior as the string grows because each concatenation may copy the accumulated content. This differs from unnecessary data copying (Category 6): the copying is an implicit side effect of the chosen string-building method. Prefer builders, buffers, or `join`-style primitives when assembling many parts.</t>
+  </si>
+  <si>
+    <t>Example: `s = s + part` inside a loop over many parts, instead of collecting parts and using `''.join(parts)` (or an equivalent string builder).</t>
+  </si>
+  <si>
+    <t>C10.S5</t>
+  </si>
+  <si>
+    <t>Defining a variable either local or global can be inefficient depending on the context. Do not use when the variable must be global for correctness or module-level configuration.</t>
+  </si>
+  <si>
+    <t>Example: Repeatedly reading a global constant in a tight Python loop instead of binding it to a local variable once before the loop.</t>
+  </si>
+  <si>
+    <t>C10.S6</t>
+  </si>
+  <si>
+    <t>Uses expensive functions or logic to compute results that are constant, precomputable, or trivially derivable. The hallmark is calling heavyweight routines for values that do not depend on runtime inputs (or depend only on a small finite set). Do not use when the value truly depends on runtime data or must be computed for correctness.</t>
+  </si>
+  <si>
+    <t>Example: Using expensive function for constants or use modulo (%) instead of conditional</t>
+  </si>
+  <si>
+    <t>C10.S7</t>
+  </si>
+  <si>
+    <t>Uses operator syntax (e.g., `+`, `*`, `==`) on non-primitive or user-defined types where the operator triggers an overloaded method that allocates objects or performs heavy computation. The smell is that the code *looks* like a cheap primitive operation, but it actually performs dynamic dispatch and potentially large memory traffic, especially inside loops. Prefer in-place operators, specialized APIs, or bulk primitives when they avoid allocations or repeated dispatch.</t>
+  </si>
+  <si>
+    <t>Example: having Obj A; Obj B and In a tight loop, using A + B which adds a lot of computation</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>Energy waste driven by CPU/memory hierarchy behavior such as cache locality, branch prediction, and data layout. These smells are about how data and control flow interact with the hardware (or VM) rather than high-level algorithm choice. Use this category when profiling indicates cache misses, poor locality, or branch mispredictions dominate runtime.</t>
+  </si>
+  <si>
+    <t>C11.S1</t>
+  </si>
+  <si>
+    <t>Traverses arrays/matrices with a stride pattern that causes frequent cache misses, such as visiting columns in a row-major layout. The hallmark is regular but poorly ordered access that defeats spatial locality. Do not use when data is inherently stored in that layout due to interoperability constraints.</t>
+  </si>
+  <si>
+    <t>Example: Accessing a 2D array column-by-column in a language/runtime that stores rows contiguously, causing many cache misses.</t>
+  </si>
+  <si>
+    <t>C11.S2</t>
+  </si>
+  <si>
+    <t>Touches a small scattered subset inside a large structure repeatedly, preventing effective caching and locality. The hallmark is pointer chasing or non-contiguous access patterns driven by sparse indices or indirection-heavy structures. Do not use when the data is inherently sparse and alternative representations are impossible.</t>
+  </si>
+  <si>
+    <t>Example: Repeatedly accessing random indices of a huge array in a tight loop, or walking a pointer-heavy structure that jumps around memory.</t>
+  </si>
+  <si>
+    <t>C11.S3</t>
+  </si>
+  <si>
+    <t>Uses highly data-dependent branching patterns in tight loops that defeat branch prediction. The hallmark is frequent mispredictions causing pipeline flushes and wasted CPU cycles. Do not use when branching is required for correctness and cannot be transformed (e.g., via predication or data layout changes).</t>
+  </si>
+  <si>
+    <t>Example: A tight loop with an if-statement whose condition is essentially random across iterations, causing frequent branch mispredictions.</t>
+  </si>
+  <si>
+    <t>C11.S4</t>
+  </si>
+  <si>
+    <t>Example: You declare a rarely accessed "error_logging" array at the very top of your function, unintentionally granting it the most energy-efficient "offset 0" memory address.</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>Energy waste due to thread/task misuse, synchronization overhead, contention, or forced serialization. This category includes excess locking, background work that never stops, and architectures that prevent parallelism benefits. Use it when multiple execution contexts are involved and waiting/wakeups or serialized bottlenecks dominate.</t>
+  </si>
+  <si>
+    <t>C12.S1</t>
+  </si>
+  <si>
+    <t>Uses heavyweight synchronization too frequently or on overly broad critical sections, leading to contention and context switching. The hallmark is threads spending significant time waiting on locks rather than doing useful work. This differs from forced serial bottlenecks: contention can happen even when parallelism is intended. Do not use when the critical section must be serialized for correctness and is tiny and infrequent.</t>
+  </si>
+  <si>
+    <t>Example: Guarding a frequently updated counter with a global lock across many threads instead of using a more scalable approach.</t>
+  </si>
+  <si>
+    <t>C12.S2</t>
+  </si>
+  <si>
+    <t>Architecture forces “single-file” execution (single shared resource, global queue, central lock) that cancels parallelism benefits. The signal is that concurrency exists but work is effectively serialized by design. This differs from contended locking, here the bottleneck is structural even if contention is reduced. Do not use when the workload is not parallelizable by nature.</t>
+  </si>
+  <si>
+    <t>Example: A pipeline with many worker threads that all must pass through one single-threaded stage, dominating total runtime.</t>
+  </si>
+  <si>
+    <t>C12.S3</t>
+  </si>
+  <si>
+    <t>Starts threads/tasks that are never stopped, joined, or allowed to sleep appropriately, consuming energy indefinitely. Signals include runaway background loops, busy-waiting, or periodic timers that keep firing without need. Do not use when a daemon truly must run continuously and its overhead is measured and acceptable.</t>
+  </si>
+  <si>
+    <t>Example: Spawning a background thread per request and never terminating it, leading to many idle threads consuming resources.</t>
+  </si>
+  <si>
+    <t>C12.S4</t>
+  </si>
+  <si>
+    <t>Performs long-running CPU or I/O tasks on the main event/UI thread, causing stalls and preventing idle/sleep states. This often triggers extra retries/timeouts or additional redraw work, compounding energy cost. Do not use when no UI/main-thread constraints exist (then classify under compute or I/O categories).</t>
+  </si>
+  <si>
+    <t>Example: Running a large database query or image processing on a mobile UI thread, freezing the interface and preventing efficient power management.</t>
+  </si>
+  <si>
+    <t>C12.S5</t>
+  </si>
+  <si>
+    <t>Executes work serially even though tasks are independent and could run concurrently without violating correctness, leading to longer CPU active time and higher energy use. The smell is not about contention; it is about leaving parallelism unused where it would reduce wall-clock time or allow earlier idle/sleep states.</t>
+  </si>
+  <si>
+    <t>Example: Processing many independent images/files one-by-one on a multi-core system when a bounded worker pool could process them in parallel.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2047,16 +2729,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7EEF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -2064,14 +2773,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6919,4 +7664,1535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E156957B-EDA9-4BF1-9497-AC41212BE764}">
+  <dimension ref="A1:F78"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="110" customWidth="1"/>
+    <col min="6" max="6" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>656</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>657</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>659</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>661</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>662</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>670</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>677</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>593</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>690</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>693</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>698</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>707</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>708</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>714</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>716</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>572</v>
+      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
+        <v>718</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>616</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>730</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>734</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>739</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>740</v>
+      </c>
+      <c r="F31" s="3"/>
+    </row>
+    <row r="32" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>741</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>742</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>744</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>745</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>748</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
+        <v>750</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>751</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="F36" s="3"/>
+    </row>
+    <row r="37" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>756</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>758</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
+        <v>760</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>763</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>764</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
+        <v>772</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>753</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>588</v>
+      </c>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="F44" s="3"/>
+    </row>
+    <row r="45" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>777</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>778</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>784</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>786</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>787</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>790</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>581</v>
+      </c>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="F51" s="3"/>
+    </row>
+    <row r="52" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>798</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>609</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>582</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="F56" s="3"/>
+    </row>
+    <row r="57" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
+        <v>811</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>597</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="5" t="s">
+        <v>817</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="F60" s="3"/>
+    </row>
+    <row r="61" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>823</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>826</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="F63" s="5" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
+        <v>834</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="D65" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>835</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>838</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>840</v>
+      </c>
+      <c r="B67" t="s">
+        <v>658</v>
+      </c>
+      <c r="C67" t="s">
+        <v>635</v>
+      </c>
+      <c r="D67" t="s">
+        <v>820</v>
+      </c>
+      <c r="E67" t="s">
+        <v>841</v>
+      </c>
+      <c r="F67" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>637</v>
+      </c>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="F68" s="3"/>
+    </row>
+    <row r="69" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
+        <v>845</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="5" t="s">
+        <v>848</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>849</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>852</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>623</v>
+      </c>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3" t="s">
+        <v>857</v>
+      </c>
+      <c r="F73" s="3"/>
+    </row>
+    <row r="74" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="5" t="s">
+        <v>858</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>856</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="D75" s="5" t="s">
+        <v>856</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>862</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
+        <v>864</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="D76" s="5" t="s">
+        <v>856</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>658</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="D77" s="5" t="s">
+        <v>856</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>868</v>
+      </c>
+      <c r="F77" s="5" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>870</v>
+      </c>
+      <c r="B78" t="s">
+        <v>658</v>
+      </c>
+      <c r="C78" t="s">
+        <v>628</v>
+      </c>
+      <c r="D78" t="s">
+        <v>856</v>
+      </c>
+      <c r="E78" t="s">
+        <v>871</v>
+      </c>
+      <c r="F78" t="s">
+        <v>872</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F77" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>